<commit_message>
Added test case for failing loading https://github.com/wojciech-kwapisiewicz/MyBudget/issues/36
</commit_message>
<xml_diff>
--- a/MyBudget.OperationsLoading.Tests/Resources/BNP_TestOperations_v2.xlsx
+++ b/MyBudget.OperationsLoading.Tests/Resources/BNP_TestOperations_v2.xlsx
@@ -11,7 +11,7 @@
     <sheet name="ExcelExportFile" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">ExcelExportFile!$A$1:$L$11</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">ExcelExportFile!$A$1:$L$12</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="40">
   <si>
     <t xml:space="preserve">Data transakcji</t>
   </si>
@@ -72,6 +72,9 @@
   </si>
   <si>
     <t xml:space="preserve">Transakcja kartą</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niezrealizowana</t>
   </si>
   <si>
     <t xml:space="preserve">Zrealizowana</t>
@@ -351,8 +354,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultColWidth="8.578125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr defaultColWidth="8.58984375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.71"/>
@@ -404,11 +407,9 @@
     </row>
     <row r="2" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="n">
-        <v>43886</v>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>43886</v>
-      </c>
+        <v>43887</v>
+      </c>
+      <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="4" t="n">
         <v>-2.4</v>
@@ -436,23 +437,23 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="n">
-        <v>43884</v>
+        <v>43886</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>43885</v>
+        <v>43886</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="4" t="n">
-        <v>-234</v>
+        <v>-2.4</v>
       </c>
       <c r="E3" s="0" t="s">
         <v>12</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>14</v>
@@ -461,157 +462,155 @@
         <v>15</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>-234</v>
+        <v>-2.4</v>
       </c>
       <c r="K3" s="0" t="s">
         <v>12</v>
       </c>
       <c r="L3" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="n">
-        <v>43882</v>
+        <v>43884</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>43882</v>
+        <v>43885</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="4" t="n">
-        <v>2345</v>
+        <v>-234</v>
       </c>
       <c r="E4" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="5"/>
+      <c r="G4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>19</v>
-      </c>
       <c r="H4" s="5" t="s">
         <v>14</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>2345</v>
+        <v>-234</v>
       </c>
       <c r="K4" s="0" t="s">
         <v>12</v>
       </c>
       <c r="L4" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="n">
-        <v>43881</v>
+        <v>43882</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>43881</v>
+        <v>43882</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="4" t="n">
-        <v>-300</v>
+        <v>2345</v>
       </c>
       <c r="E5" s="0" t="s">
         <v>12</v>
       </c>
       <c r="F5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" s="0" t="s">
-        <v>23</v>
-      </c>
       <c r="J5" s="4" t="n">
-        <v>-300</v>
+        <v>2345</v>
       </c>
       <c r="K5" s="0" t="s">
         <v>12</v>
       </c>
       <c r="L5" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="n">
-        <v>43880</v>
+        <v>43881</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>43880</v>
+        <v>43881</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="4" t="n">
-        <v>-150</v>
+        <v>-300</v>
       </c>
       <c r="E6" s="0" t="s">
         <v>12</v>
       </c>
       <c r="F6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I6" s="0" t="s">
-        <v>26</v>
-      </c>
       <c r="J6" s="4" t="n">
-        <v>-150</v>
+        <v>-300</v>
       </c>
       <c r="K6" s="0" t="s">
         <v>12</v>
       </c>
       <c r="L6" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="58.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="n">
-        <v>43878</v>
+        <v>43880</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>43878</v>
+        <v>43880</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="4" t="n">
-        <v>-1000</v>
+        <v>-150</v>
       </c>
       <c r="E7" s="0" t="s">
         <v>12</v>
       </c>
       <c r="F7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I7" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="G7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I7" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="J7" s="4" t="n">
-        <v>-1000</v>
+        <v>-150</v>
       </c>
       <c r="K7" s="0" t="s">
         <v>12</v>
       </c>
       <c r="L7" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="58.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -623,139 +622,175 @@
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="4" t="n">
-        <v>-1200</v>
+        <v>-1000</v>
       </c>
       <c r="E8" s="0" t="s">
         <v>12</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I8" s="0" t="s">
-        <v>31</v>
-      </c>
       <c r="J8" s="4" t="n">
-        <v>-1200</v>
+        <v>-1000</v>
       </c>
       <c r="K8" s="0" t="s">
         <v>12</v>
       </c>
       <c r="L8" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="58.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="n">
-        <v>43877</v>
+        <v>43878</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>43877</v>
+        <v>43878</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="4" t="n">
-        <v>50</v>
+        <v>-1200</v>
       </c>
       <c r="E9" s="0" t="s">
         <v>12</v>
       </c>
       <c r="F9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="G9" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I9" s="0" t="s">
-        <v>34</v>
-      </c>
       <c r="J9" s="4" t="n">
-        <v>50</v>
+        <v>-1200</v>
       </c>
       <c r="K9" s="0" t="s">
         <v>12</v>
       </c>
       <c r="L9" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="n">
-        <v>43872</v>
+        <v>43877</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>43872</v>
+        <v>43877</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="4" t="n">
-        <v>-300</v>
+        <v>50</v>
       </c>
       <c r="E10" s="0" t="s">
         <v>12</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G10" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="H10" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I10" s="0" t="s">
-        <v>34</v>
-      </c>
       <c r="J10" s="4" t="n">
-        <v>-300</v>
+        <v>50</v>
       </c>
       <c r="K10" s="0" t="s">
         <v>12</v>
       </c>
       <c r="L10" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="n">
-        <v>43871</v>
+        <v>43872</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>43871</v>
+        <v>43872</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="4" t="n">
+        <v>-300</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I11" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>-300</v>
+      </c>
+      <c r="K11" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="L11" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="n">
+        <v>43871</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>43871</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="4" t="n">
         <v>-120</v>
       </c>
-      <c r="E11" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G11" s="5" t="s">
+      <c r="E12" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="H11" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I11" s="0" t="s">
+      <c r="G12" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="H12" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I12" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="J12" s="4" t="n">
         <v>-120</v>
       </c>
-      <c r="K11" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="L11" s="0" t="s">
-        <v>16</v>
+      <c r="K12" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="L12" s="0" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>